<commit_message>
The consistency gate could not read the one deliverable the judges open as a file
docs/Vero7878_track2_methods.xlsx is the organizers' methods form and a submitted
deliverable, and nothing checked it: it is a zip, so read_text returned binary noise
and every count regex matched nothing. The moment the gate could read it, it was
carrying three errors.

It said "36 claims: 18 mechanism, 11 regulatory" after the ledger had grown to 37/12.
It said "35 load-bearing PMIDs" against 36. And it still said the EMA non-renewal of
ataluren "closes the readthrough route for the truncating allele" — the global negative
withdrawn in the previous commit, now replaced with the bounded per-patient statement
and the Great Britain counterexample.

The gate now extracts the workbook's cell text and runs the same count and denominator
checks over it, and a new perturbation test retypes a count inside the .xlsx and
requires the block, so this cannot be a one-off repair. Suite 76 -> 77.
</commit_message>
<xml_diff>
--- a/docs/Vero7878_track2_methods.xlsx
+++ b/docs/Vero7878_track2_methods.xlsx
@@ -542,9 +542,9 @@
         <is>
           <t>Mechanism-first, falsification-first, and audited.
 Curation. Each lead was sent to an independent adversarial review instructed to REFUTE it, not to support it. A single-standard re-score was then applied to remove survivorship bias. One consequence worth naming: our earlier lead candidate, 4-PBA, was demoted to INSUFFICIENT on mechanism (its action is secretory-cargo export via COPII sorting, not cytosolic chaperoning, with zero BUBR1-specific data), and that demotion is carried consistently across report, pitch, candidate table and submission record.
-Citation discipline. Every load-bearing citation is resolved against Europe PMC by scripts/phase1/16_verify_citations.py, which compares the returned title with the one we recorded. 35 load-bearing PMIDs, zero unresolved mismatches. A separate human verification pass re-read the primary texts and is recorded with its own access limits in registers/citation_manual_check_2026-10-19b.md. That pass removed one miscited source from the mechanism chain and downgraded one edge from 'measured' to 'asserted' because the source's human result is the authors' stated prediction, not a measurement.
+Citation discipline. Every load-bearing citation is resolved against Europe PMC by scripts/phase1/16_verify_citations.py, which compares the returned title with the one we recorded. 36 load-bearing PMIDs, zero unresolved mismatches. A separate human verification pass re-read the primary texts and is recorded with its own access limits in registers/citation_manual_check_2026-10-19b.md. That pass removed one miscited source from the mechanism chain and downgraded one edge from 'measured' to 'asserted' because the source's human result is the authors' stated prediction, not a measurement.
 One citation is carried at a strength we would normally reject, and we flag it rather than hide it: for the SIRT2-K250 link the publisher deposited no abstract and we could not obtain the full text, so it is graded 'asserted', cited for direction only, and no result is quoted from it. We judged that disclosing a load-bearing COUNTER-argument we could not fully verify was better than omitting the counter-argument.
-Claim ledger. Every statement that affects the conclusion has a row in registers/claim_ledger.csv (36 claims: 18 mechanism, 11 regulatory, 5 global-negative, 2 method), each with source URL, locator, checked date, evidence strength, counter-evidence and disposition. The ledger is GENERATED from the mechanism chain and the eligibility matrix on every clean run, not hand-maintained, so a claim cannot drift away from its source. The five global-negative claims — the 'no approved drug does X' statements that one counterexample would destroy — each carry a dated, reproducible search in registers/search_strategies.md with the verbatim query, the hits, and why each hit does not count.</t>
+Claim ledger. Every statement that affects the conclusion has a row in registers/claim_ledger.csv (37 claims: 18 mechanism, 12 regulatory, 5 global-negative, 2 method), each with source URL, locator, checked date, evidence strength, counter-evidence and disposition. The ledger is GENERATED from the mechanism chain and the eligibility matrix on every clean run, not hand-maintained, so a claim cannot drift away from its source. The five global-negative claims — the 'no approved drug does X' statements that one counterexample would destroy — each carry a dated, reproducible search in registers/search_strategies.md with the verbatim query, the hits, and why each hit does not count.</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
         <is>
           <t>Regulatory / product level
 - DailyMed (FDA Structured Product Labels) — the load-bearing source for product eligibility. Labels opened and quoted verbatim with their revision dates, including niacin extended-release (setid 6e604319-e164-4056-ab80-b78b98c519c7, revised 12/2025), niacin immediate-release (Niacor), Buphenyl, Ravicti, Acetadote, sirolimus, metformin.
-- EMA EPAR — Translarna (ataluren): conditional marketing authorisation NOT renewed on 28 March 2025 because effectiveness was not confirmed. This closes the readthrough route for the truncating allele.
+- EMA EPAR — Translarna (ataluren): conditional marketing authorisation NOT renewed on 28 March 2025 because effectiveness was not confirmed. We first read this as closing the readthrough route; it does not. Ataluren retains a Great Britain marketing authorisation (live UK SmPC, 250 mg dated 2026-03-31, checked 2026-10-20), for a different gene and indication, so the bounded statement is that no approved readthrough agent is eligible for this allele rather than that none exists.
 - NIH Office of Dietary Supplements — for NMN and NR, which are supplements rather than approved drugs. These rows are marked in the matrix as landing pages with no product label, because the ABSENCE of a label is exactly what the row records.
 Target / tractability
 - Open Targets Platform, target ENSG00000156970 (BUB1B), data version 26.09, queried 2026-10-19 — tractability across small molecule, antibody, PROTAC and other-clinical modalities.

</xml_diff>